<commit_message>
Redesign BUS331 investment project workflow
</commit_message>
<xml_diff>
--- a/files/BUS331_Investment_Committee_Decision_Record_Student.xlsx
+++ b/files/BUS331_Investment_Committee_Decision_Record_Student.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="START HERE" sheetId="1" r:id="Re5d9bb9fc6394467"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMMITTEE ROSTER" sheetId="2" r:id="Rcf5eb79eba084c63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ANALYST DECISION LOG" sheetId="3" r:id="Rcf54d98cd75449b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PHASE 1" sheetId="4" r:id="R07842bd965ca4690"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PHASE 2 CLIENT 1" sheetId="5" r:id="R0b2893e44b3a4b14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PHASE 2 CLIENT 2" sheetId="6" r:id="R903d9252853245b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PHASE 2 CLIENT 3" sheetId="7" r:id="Rd7ba186e58af45a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PHASE 3" sheetId="8" r:id="R9bed630886b9475c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI AUDIT LOG" sheetId="9" r:id="R7ebd1a91354543e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="START HERE" sheetId="1" r:id="rId4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMMITTEE ROSTER" sheetId="2" r:id="rId5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ANALYST DECISION LOG" sheetId="3" r:id="rId6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PHASE 1" sheetId="4" r:id="rId7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PHASE 2 CLIENT 1" sheetId="5" r:id="rId8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PHASE 2 CLIENT 2" sheetId="6" r:id="rId9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PHASE 2 CLIENT 3" sheetId="7" r:id="rId10"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PHASE 3" sheetId="8" r:id="rId11"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI AUDIT LOG" sheetId="9" r:id="rId12"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1410,10 +1410,10 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="14" t="str">
-        <x:v>AI interview + challenge</x:v>
+        <x:v>Alternative + trade-off</x:v>
       </x:c>
       <x:c r="B8" s="16" t="str">
-        <x:v>Summarize the bounded client interview and the strongest counterargument; do not paste a transcript as analysis.</x:v>
+        <x:v>Record the strongest realistic alternative rejected and the key trade-off behind the recommendation. Portfolio Manager entries record integration choices; Risk and Derivatives entries record residual risk and hedge/no-hedge evidence.</x:v>
       </x:c>
       <x:c r="C8" s="16" t="str"/>
       <x:c r="D8" s="16" t="str"/>
@@ -1641,7 +1641,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>Assign one student to each committee seat. Roles define leadership; all members share the final decision.</x:v>
+        <x:v>Assign one student to each of five committee seats. Roles define distinct decision rights; all members share the final decision.</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -1709,38 +1709,56 @@
     </x:row>
     <x:row r="7" ht="72" customHeight="1">
       <x:c r="A7" s="52" t="str">
-        <x:v>Fund and ETF Analyst</x:v>
+        <x:v>Equity Analyst</x:v>
       </x:c>
       <x:c r="B7" s="53" t="str"/>
       <x:c r="C7" s="54" t="str">
-        <x:v>Own pooled-vehicle due diligence, diversification, benchmark fit, fees, liquidity, tax considerations, and active-versus-passive implementation.</x:v>
+        <x:v>Own equity-fund and ETF due diligence and the limited use of individual equities, including exposure, style, sector, holdings, costs, liquidity, overlap, idiosyncratic risk, and position-size evidence.</x:v>
       </x:c>
       <x:c r="D7" s="54" t="str">
-        <x:v>Identify the client's diversification, access, liquidity, cost, tax, values, and vehicle requirements before screening products.</x:v>
+        <x:v>Translate the client's growth needs, time horizon, values, tax position, liquidity, and concentration limits into equity-selection guardrails.</x:v>
       </x:c>
       <x:c r="E7" s="54" t="str">
-        <x:v>Evaluate funds and ETFs using objective, holdings, benchmark, fees, liquidity, tax efficiency, and tracking evidence.</x:v>
+        <x:v>Recommend equity funds and ETFs as the primary equity vehicles and analyze any limited individual equities, including rationale, idiosyncratic risk, and position size.</x:v>
       </x:c>
       <x:c r="F7" s="54" t="str">
-        <x:v>Defend vehicle selection, implementation feasibility, diversification, and product-level due diligence.</x:v>
+        <x:v>Defend equity exposures, vehicle choices, limited individual-security decisions, rejected alternatives, and their client fit.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="72" customHeight="1">
       <x:c r="A8" s="52" t="str">
-        <x:v>Portfolio Manager and Risk Analyst</x:v>
+        <x:v>Portfolio Manager</x:v>
       </x:c>
       <x:c r="B8" s="53" t="str"/>
       <x:c r="C8" s="54" t="str">
-        <x:v>Own portfolio integration, risk capacity versus willingness, the drawdown tripwire, decision-log quality, stress testing, and mandate-breach escalation.</x:v>
+        <x:v>Own portfolio integration: resolve overlap and concentration, set final selection and weights, record explicit trade-offs, maintain decision-log quality, and move the integrated recommendation to a vote.</x:v>
       </x:c>
       <x:c r="D8" s="54" t="str">
-        <x:v>Reconcile risk capacity and willingness, set provisional portfolio guardrails, challenge assumptions, and audit the Analyst Decision Log.</x:v>
+        <x:v>Reconcile risk capacity and willingness, set provisional portfolio guardrails, coordinate the committee challenge, and audit the Analyst Decision Log.</x:v>
       </x:c>
       <x:c r="E8" s="54" t="str">
-        <x:v>Integrate the allocation, run bear-case stress tests, compare mitigants, identify breaches, and require corrective action.</x:v>
+        <x:v>Integrate analyst recommendations, resolve duplication and concentration, choose the final 8–10 holdings and weights, and record the trade-offs behind every integration decision.</x:v>
       </x:c>
       <x:c r="F8" s="54" t="str">
-        <x:v>State the integrated recommendation, present the strongest downside case, and lead preparation for adversarial Q&amp;A.</x:v>
+        <x:v>State and defend the integrated recommendation, portfolio construction decisions, final weights, rejected integrations, and implementation priorities.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="72" customHeight="1">
+      <x:c r="A9" s="52" t="str">
+        <x:v>Risk and Derivatives Analyst</x:v>
+      </x:c>
+      <x:c r="B9" s="53" t="str"/>
+      <x:c r="C9" s="54" t="str">
+        <x:v>Own portfolio-level risk diagnosis, stress testing, residual-risk evidence, mandate-breach escalation, and the hedge or no-hedge conclusion; do not manufacture a derivative position when no targeted hedge is justified.</x:v>
+      </x:c>
+      <x:c r="D9" s="54" t="str">
+        <x:v>Define the downside questions, drawdown tripwire, stress priorities, and residual-risk evidence the final portfolio must address.</x:v>
+      </x:c>
+      <x:c r="E9" s="54" t="str">
+        <x:v>Run portfolio-level stress tests, identify residual risk, and document either one targeted hedge or a fully supported no-hedge conclusion, including cost, liquidity, trade-offs, residual risk, and adjustment or removal conditions.</x:v>
+      </x:c>
+      <x:c r="F9" s="54" t="str">
+        <x:v>Defend the stress evidence, residual risk, hedge or no-hedge decision, limits of the analysis, and conditions that would change the risk response.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="23" customHeight="1">
@@ -1880,7 +1898,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>Human-first judgment → AI interview and challenge → human verification → final reasoning → downstream guardrail</x:v>
+        <x:v>Recommendation → alternative rejected → key trade-off → verification → final reasoning → downstream guardrail</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -1904,7 +1922,7 @@
     </x:row>
     <x:row r="4" ht="30" customHeight="1">
       <x:c r="A4" s="58" t="str">
-        <x:v>Before using AI, each of the four roles records at least one initial judgment for each assigned client. Minimum Phase 1 evidence: 12 complete role-by-client entries across the team.</x:v>
+        <x:v>Each of the five roles records at least one recommendation for each assigned client. Every material entry includes an alternative rejected and a key trade-off. Minimum Phase 1 evidence: 15 complete role-by-client entries across the team.</x:v>
       </x:c>
       <x:c r="B4" s="58"/>
       <x:c r="C4" s="58"/>
@@ -1998,10 +2016,10 @@
         <x:v>Claim type</x:v>
       </x:c>
       <x:c r="I7" s="21" t="str">
-        <x:v>AI challenge prompt / purpose</x:v>
+        <x:v>Alternative(s) rejected</x:v>
       </x:c>
       <x:c r="J7" s="21" t="str">
-        <x:v>AI output summary</x:v>
+        <x:v>Key trade-off</x:v>
       </x:c>
       <x:c r="K7" s="21" t="str">
         <x:v>Claim to verify</x:v>
@@ -2829,13 +2847,13 @@
         <x:v>Minimum required</x:v>
       </x:c>
       <x:c r="H40" s="57" t="n">
-        <x:v>12</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="J40" s="25" t="str">
         <x:v>Log readiness</x:v>
       </x:c>
       <x:c r="K40" s="100" t="str">
-        <x:f>IF(OR(E6="",H6="",K6=""),"ENTER 3 CLIENTS",IF(COUNTIF(B47:D50,"READY")&lt;H40,"COVERAGE INCOMPLETE",IF(COUNTIF(T8:T37,"INCOMPLETE")+E40&gt;0,"REVIEW LOG","READY FOR PHASE 1 GATE")))</x:f>
+        <x:f>IF(OR(E6="",H6="",K6=""),"ENTER 3 CLIENTS",IF(COUNTIF(B47:D51,"READY")&lt;H40,"COVERAGE INCOMPLETE",IF(COUNTIF(T8:T37,"INCOMPLETE")+E40&gt;0,"REVIEW LOG","READY FOR PHASE 1 GATE")))</x:f>
         <x:v>ENTER 3 CLIENTS</x:v>
       </x:c>
       <x:c r="L40" s="101"/>
@@ -2843,7 +2861,7 @@
     </x:row>
     <x:row r="42" ht="34" customHeight="1">
       <x:c r="A42" s="104" t="str">
-        <x:v>Evidence-ready means the entry shows the initial judgment, the AI challenge, a human-verified source and as-of date, what changed, the final reasoning, a downstream guardrail, and peer review. Contradicted or unverifiable material claims must be revised or carried to the committee as an explicit open issue.</x:v>
+        <x:v>Evidence-ready means the entry shows the recommendation or initial judgment, an alternative rejected, a key trade-off, a human-verified source and as-of date, what changed, the final reasoning, a downstream guardrail, and peer review. Portfolio Manager entries identify integration decisions; Risk and Derivatives entries identify residual risk and hedge/no-hedge evidence. Contradicted or unverifiable material claims must be revised or carried to the committee as an explicit open issue.</x:v>
       </x:c>
       <x:c r="B42" s="104"/>
       <x:c r="C42" s="104"/>
@@ -2950,7 +2968,7 @@
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="52" t="str">
-        <x:v>Fund and ETF Analyst</x:v>
+        <x:v>Equity Analyst</x:v>
       </x:c>
       <x:c r="B49" s="107" t="str">
         <x:f>IF(OR($E$6="",COUNTIFS($C$8:$C$37,$E$6,$D$8:$D$37,$A49,$T$8:$T$37,"EVIDENCE READY")=0),"MISSING","READY")</x:f>
@@ -2971,7 +2989,7 @@
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="52" t="str">
-        <x:v>Portfolio Manager and Risk Analyst</x:v>
+        <x:v>Portfolio Manager</x:v>
       </x:c>
       <x:c r="B50" s="107" t="str">
         <x:f>IF(OR($E$6="",COUNTIFS($C$8:$C$37,$E$6,$D$8:$D$37,$A50,$T$8:$T$37,"EVIDENCE READY")=0),"MISSING","READY")</x:f>
@@ -2990,9 +3008,30 @@
         <x:v>MISSING</x:v>
       </x:c>
     </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="52" t="str">
+        <x:v>Risk and Derivatives Analyst</x:v>
+      </x:c>
+      <x:c r="B51" s="107" t="str">
+        <x:f>IF(OR($E$6="",COUNTIFS($C$8:$C$37,$E$6,$D$8:$D$37,$A51,$T$8:$T$37,"EVIDENCE READY")=0),"MISSING","READY")</x:f>
+        <x:v>MISSING</x:v>
+      </x:c>
+      <x:c r="C51" s="107" t="str">
+        <x:f>IF(OR($H$6="",COUNTIFS($C$8:$C$37,$H$6,$D$8:$D$37,$A51,$T$8:$T$37,"EVIDENCE READY")=0),"MISSING","READY")</x:f>
+        <x:v>MISSING</x:v>
+      </x:c>
+      <x:c r="D51" s="107" t="str">
+        <x:f>IF(OR($K$6="",COUNTIFS($C$8:$C$37,$K$6,$D$8:$D$37,$A51,$T$8:$T$37,"EVIDENCE READY")=0),"MISSING","READY")</x:f>
+        <x:v>MISSING</x:v>
+      </x:c>
+      <x:c r="E51" s="107" t="str">
+        <x:f>IF(COUNTIF(B51:D51,"MISSING")&gt;0,"MISSING","READY")</x:f>
+        <x:v>MISSING</x:v>
+      </x:c>
+    </x:row>
     <x:row r="52" ht="30" customHeight="1">
       <x:c r="A52" s="104" t="str">
-        <x:v>The Phase 1 gate remains closed until every role has at least one evidence-ready entry for each of the three assigned clients. The client names in row 6 must match the Client column exactly.</x:v>
+        <x:v>The Phase 1 gate remains closed until every one of the five roles has at least one evidence-ready entry for each of the three assigned clients. The client names in row 6 must match the Client column exactly.</x:v>
       </x:c>
       <x:c r="B52" s="104"/>
       <x:c r="C52" s="104"/>
@@ -3050,7 +3089,7 @@
     <x:cfRule type="containsText" dxfId="25" priority="13" operator="containsText" text="MISSING"/>
     <x:cfRule type="containsText" dxfId="26" priority="14" operator="containsText" text="ENTER"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="B47:E50">
+  <x:conditionalFormatting sqref="B47:E51">
     <x:cfRule type="containsText" dxfId="27" priority="15" operator="containsText" text="EVIDENCE READY"/>
     <x:cfRule type="containsText" dxfId="28" priority="16" operator="containsText" text="REVISE"/>
     <x:cfRule type="containsText" dxfId="29" priority="17" operator="containsText" text="INCOMPLETE"/>
@@ -3061,7 +3100,7 @@
   </x:conditionalFormatting>
   <x:dataValidations count="5">
     <x:dataValidation type="list" sqref="D8:D37">
-      <x:formula1>"Client and Macro Strategist,Fixed-Income Analyst,Fund and ETF Analyst,Portfolio Manager and Risk Analyst"</x:formula1>
+      <x:formula1>"Client and Macro Strategist,Fixed-Income Analyst,Equity Analyst,Portfolio Manager,Risk and Derivatives Analyst"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="G8:G37">
       <x:formula1>"Low,Medium,High"</x:formula1>
@@ -3108,7 +3147,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>Frame the Mandate | All four committee members review, vote, and sign this record.</x:v>
+        <x:v>Frame the Mandate | All five committee members review, vote, and sign this record.</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -3361,7 +3400,7 @@
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="114" t="str">
-        <x:v>Fund &amp; ETF</x:v>
+        <x:v>Equity</x:v>
       </x:c>
       <x:c r="B27" s="85" t="str"/>
       <x:c r="C27" s="86" t="str"/>
@@ -3372,21 +3411,32 @@
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="114" t="str">
-        <x:v>Portfolio &amp; Risk</x:v>
-      </x:c>
-      <x:c r="B28" s="88" t="str"/>
-      <x:c r="C28" s="89" t="str"/>
-      <x:c r="D28" s="89" t="str"/>
-      <x:c r="E28" s="89" t="str"/>
-      <x:c r="F28" s="89" t="str"/>
-      <x:c r="G28" s="90" t="str"/>
+        <x:v>Portfolio Manager</x:v>
+      </x:c>
+      <x:c r="B28" s="85" t="str"/>
+      <x:c r="C28" s="86" t="str"/>
+      <x:c r="D28" s="86" t="str"/>
+      <x:c r="E28" s="86" t="str"/>
+      <x:c r="F28" s="86" t="str"/>
+      <x:c r="G28" s="87" t="str"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="114" t="str">
+        <x:v>Risk &amp; Derivatives</x:v>
+      </x:c>
+      <x:c r="B29" s="88" t="str"/>
+      <x:c r="C29" s="89" t="str"/>
+      <x:c r="D29" s="89" t="str"/>
+      <x:c r="E29" s="89" t="str"/>
+      <x:c r="F29" s="89" t="str"/>
+      <x:c r="G29" s="90" t="str"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="25" t="str">
         <x:v>Decision status</x:v>
       </x:c>
       <x:c r="B30" s="28" t="str">
-        <x:f>IF(COUNTIF(C25:C28,"Revise")+COUNTIF(C25:C28,"Reject")&gt;0,"REVISION REQUIRED",IF(COUNTIF(C25:C28,"Approve")=4,"APPROVED","INCOMPLETE"))</x:f>
+        <x:f>IF(COUNTIF(C25:C29,"Revise")+COUNTIF(C25:C29,"Reject")&gt;0,"REVISION REQUIRED",IF(COUNTIF(C25:C29,"Approve")=5,"APPROVED","INCOMPLETE"))</x:f>
         <x:v>INCOMPLETE</x:v>
       </x:c>
       <x:c r="C30" s="29"/>
@@ -3513,7 +3563,7 @@
     </x:row>
     <x:row r="44" ht="32" customHeight="1">
       <x:c r="A44" s="104" t="str">
-        <x:v>Approval requires four Approve votes. Any Revise or Reject vote produces REVISION REQUIRED; document the change and reconvene before the next gate.</x:v>
+        <x:v>Approval requires five Approve votes. Any Revise or Reject vote produces REVISION REQUIRED; document the change and reconvene before the next gate.</x:v>
       </x:c>
       <x:c r="B44" s="104"/>
       <x:c r="C44" s="104"/>
@@ -3553,7 +3603,7 @@
     <x:dataValidation type="list" sqref="G10:G15">
       <x:formula1>"Not reviewed,Reviewed,Needs follow-up"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="C25:C28">
+    <x:dataValidation type="list" sqref="C25:C29">
       <x:formula1>"Approve,Revise,Reject"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="E38:E42">
@@ -3592,7 +3642,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>Build &amp; Challenge | All four committee members review, vote, and sign this record.</x:v>
+        <x:v>Build &amp; Challenge | All five committee members review, vote, and sign this record.</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -3845,7 +3895,7 @@
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="114" t="str">
-        <x:v>Fund &amp; ETF</x:v>
+        <x:v>Equity</x:v>
       </x:c>
       <x:c r="B27" s="85" t="str"/>
       <x:c r="C27" s="86" t="str"/>
@@ -3856,21 +3906,32 @@
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="114" t="str">
-        <x:v>Portfolio &amp; Risk</x:v>
-      </x:c>
-      <x:c r="B28" s="88" t="str"/>
-      <x:c r="C28" s="89" t="str"/>
-      <x:c r="D28" s="89" t="str"/>
-      <x:c r="E28" s="89" t="str"/>
-      <x:c r="F28" s="89" t="str"/>
-      <x:c r="G28" s="90" t="str"/>
+        <x:v>Portfolio Manager</x:v>
+      </x:c>
+      <x:c r="B28" s="85" t="str"/>
+      <x:c r="C28" s="86" t="str"/>
+      <x:c r="D28" s="86" t="str"/>
+      <x:c r="E28" s="86" t="str"/>
+      <x:c r="F28" s="86" t="str"/>
+      <x:c r="G28" s="87" t="str"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="114" t="str">
+        <x:v>Risk &amp; Derivatives</x:v>
+      </x:c>
+      <x:c r="B29" s="88" t="str"/>
+      <x:c r="C29" s="89" t="str"/>
+      <x:c r="D29" s="89" t="str"/>
+      <x:c r="E29" s="89" t="str"/>
+      <x:c r="F29" s="89" t="str"/>
+      <x:c r="G29" s="90" t="str"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="25" t="str">
         <x:v>Decision status</x:v>
       </x:c>
       <x:c r="B30" s="28" t="str">
-        <x:f>IF(COUNTIF(C25:C28,"Revise")+COUNTIF(C25:C28,"Reject")&gt;0,"REVISION REQUIRED",IF(COUNTIF(C25:C28,"Approve")=4,"APPROVED","INCOMPLETE"))</x:f>
+        <x:f>IF(COUNTIF(C25:C29,"Revise")+COUNTIF(C25:C29,"Reject")&gt;0,"REVISION REQUIRED",IF(COUNTIF(C25:C29,"Approve")=5,"APPROVED","INCOMPLETE"))</x:f>
         <x:v>INCOMPLETE</x:v>
       </x:c>
       <x:c r="C30" s="29"/>
@@ -3997,7 +4058,7 @@
     </x:row>
     <x:row r="44" ht="32" customHeight="1">
       <x:c r="A44" s="104" t="str">
-        <x:v>Approval requires four Approve votes. Any Revise or Reject vote produces REVISION REQUIRED; document the change and reconvene before the next gate.</x:v>
+        <x:v>Approval requires five Approve votes. Any Revise or Reject vote produces REVISION REQUIRED; document the change and reconvene before the next gate.</x:v>
       </x:c>
       <x:c r="B44" s="104"/>
       <x:c r="C44" s="104"/>
@@ -4037,7 +4098,7 @@
     <x:dataValidation type="list" sqref="G10:G15">
       <x:formula1>"Not reviewed,Reviewed,Needs follow-up"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="C25:C28">
+    <x:dataValidation type="list" sqref="C25:C29">
       <x:formula1>"Approve,Revise,Reject"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="E38:E42">
@@ -4076,7 +4137,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>Build &amp; Challenge | All four committee members review, vote, and sign this record.</x:v>
+        <x:v>Build &amp; Challenge | All five committee members review, vote, and sign this record.</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -4329,7 +4390,7 @@
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="114" t="str">
-        <x:v>Fund &amp; ETF</x:v>
+        <x:v>Equity</x:v>
       </x:c>
       <x:c r="B27" s="85" t="str"/>
       <x:c r="C27" s="86" t="str"/>
@@ -4340,21 +4401,32 @@
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="114" t="str">
-        <x:v>Portfolio &amp; Risk</x:v>
-      </x:c>
-      <x:c r="B28" s="88" t="str"/>
-      <x:c r="C28" s="89" t="str"/>
-      <x:c r="D28" s="89" t="str"/>
-      <x:c r="E28" s="89" t="str"/>
-      <x:c r="F28" s="89" t="str"/>
-      <x:c r="G28" s="90" t="str"/>
+        <x:v>Portfolio Manager</x:v>
+      </x:c>
+      <x:c r="B28" s="85" t="str"/>
+      <x:c r="C28" s="86" t="str"/>
+      <x:c r="D28" s="86" t="str"/>
+      <x:c r="E28" s="86" t="str"/>
+      <x:c r="F28" s="86" t="str"/>
+      <x:c r="G28" s="87" t="str"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="114" t="str">
+        <x:v>Risk &amp; Derivatives</x:v>
+      </x:c>
+      <x:c r="B29" s="88" t="str"/>
+      <x:c r="C29" s="89" t="str"/>
+      <x:c r="D29" s="89" t="str"/>
+      <x:c r="E29" s="89" t="str"/>
+      <x:c r="F29" s="89" t="str"/>
+      <x:c r="G29" s="90" t="str"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="25" t="str">
         <x:v>Decision status</x:v>
       </x:c>
       <x:c r="B30" s="28" t="str">
-        <x:f>IF(COUNTIF(C25:C28,"Revise")+COUNTIF(C25:C28,"Reject")&gt;0,"REVISION REQUIRED",IF(COUNTIF(C25:C28,"Approve")=4,"APPROVED","INCOMPLETE"))</x:f>
+        <x:f>IF(COUNTIF(C25:C29,"Revise")+COUNTIF(C25:C29,"Reject")&gt;0,"REVISION REQUIRED",IF(COUNTIF(C25:C29,"Approve")=5,"APPROVED","INCOMPLETE"))</x:f>
         <x:v>INCOMPLETE</x:v>
       </x:c>
       <x:c r="C30" s="29"/>
@@ -4481,7 +4553,7 @@
     </x:row>
     <x:row r="44" ht="32" customHeight="1">
       <x:c r="A44" s="104" t="str">
-        <x:v>Approval requires four Approve votes. Any Revise or Reject vote produces REVISION REQUIRED; document the change and reconvene before the next gate.</x:v>
+        <x:v>Approval requires five Approve votes. Any Revise or Reject vote produces REVISION REQUIRED; document the change and reconvene before the next gate.</x:v>
       </x:c>
       <x:c r="B44" s="104"/>
       <x:c r="C44" s="104"/>
@@ -4521,7 +4593,7 @@
     <x:dataValidation type="list" sqref="G10:G15">
       <x:formula1>"Not reviewed,Reviewed,Needs follow-up"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="C25:C28">
+    <x:dataValidation type="list" sqref="C25:C29">
       <x:formula1>"Approve,Revise,Reject"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="E38:E42">
@@ -4560,7 +4632,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>Build &amp; Challenge | All four committee members review, vote, and sign this record.</x:v>
+        <x:v>Build &amp; Challenge | All five committee members review, vote, and sign this record.</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -4813,7 +4885,7 @@
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="114" t="str">
-        <x:v>Fund &amp; ETF</x:v>
+        <x:v>Equity</x:v>
       </x:c>
       <x:c r="B27" s="85" t="str"/>
       <x:c r="C27" s="86" t="str"/>
@@ -4824,21 +4896,32 @@
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="114" t="str">
-        <x:v>Portfolio &amp; Risk</x:v>
-      </x:c>
-      <x:c r="B28" s="88" t="str"/>
-      <x:c r="C28" s="89" t="str"/>
-      <x:c r="D28" s="89" t="str"/>
-      <x:c r="E28" s="89" t="str"/>
-      <x:c r="F28" s="89" t="str"/>
-      <x:c r="G28" s="90" t="str"/>
+        <x:v>Portfolio Manager</x:v>
+      </x:c>
+      <x:c r="B28" s="85" t="str"/>
+      <x:c r="C28" s="86" t="str"/>
+      <x:c r="D28" s="86" t="str"/>
+      <x:c r="E28" s="86" t="str"/>
+      <x:c r="F28" s="86" t="str"/>
+      <x:c r="G28" s="87" t="str"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="114" t="str">
+        <x:v>Risk &amp; Derivatives</x:v>
+      </x:c>
+      <x:c r="B29" s="88" t="str"/>
+      <x:c r="C29" s="89" t="str"/>
+      <x:c r="D29" s="89" t="str"/>
+      <x:c r="E29" s="89" t="str"/>
+      <x:c r="F29" s="89" t="str"/>
+      <x:c r="G29" s="90" t="str"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="25" t="str">
         <x:v>Decision status</x:v>
       </x:c>
       <x:c r="B30" s="28" t="str">
-        <x:f>IF(COUNTIF(C25:C28,"Revise")+COUNTIF(C25:C28,"Reject")&gt;0,"REVISION REQUIRED",IF(COUNTIF(C25:C28,"Approve")=4,"APPROVED","INCOMPLETE"))</x:f>
+        <x:f>IF(COUNTIF(C25:C29,"Revise")+COUNTIF(C25:C29,"Reject")&gt;0,"REVISION REQUIRED",IF(COUNTIF(C25:C29,"Approve")=5,"APPROVED","INCOMPLETE"))</x:f>
         <x:v>INCOMPLETE</x:v>
       </x:c>
       <x:c r="C30" s="29"/>
@@ -4965,7 +5048,7 @@
     </x:row>
     <x:row r="44" ht="32" customHeight="1">
       <x:c r="A44" s="104" t="str">
-        <x:v>Approval requires four Approve votes. Any Revise or Reject vote produces REVISION REQUIRED; document the change and reconvene before the next gate.</x:v>
+        <x:v>Approval requires five Approve votes. Any Revise or Reject vote produces REVISION REQUIRED; document the change and reconvene before the next gate.</x:v>
       </x:c>
       <x:c r="B44" s="104"/>
       <x:c r="C44" s="104"/>
@@ -5005,7 +5088,7 @@
     <x:dataValidation type="list" sqref="G10:G15">
       <x:formula1>"Not reviewed,Reviewed,Needs follow-up"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="C25:C28">
+    <x:dataValidation type="list" sqref="C25:C29">
       <x:formula1>"Approve,Revise,Reject"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="E38:E42">
@@ -5044,7 +5127,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>Defend the Recommendation | All four committee members review, vote, and sign this record.</x:v>
+        <x:v>Defend the Recommendation | All five committee members review, vote, and sign this record.</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -5297,7 +5380,7 @@
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="114" t="str">
-        <x:v>Fund &amp; ETF</x:v>
+        <x:v>Equity</x:v>
       </x:c>
       <x:c r="B27" s="85" t="str"/>
       <x:c r="C27" s="86" t="str"/>
@@ -5308,21 +5391,32 @@
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="114" t="str">
-        <x:v>Portfolio &amp; Risk</x:v>
-      </x:c>
-      <x:c r="B28" s="88" t="str"/>
-      <x:c r="C28" s="89" t="str"/>
-      <x:c r="D28" s="89" t="str"/>
-      <x:c r="E28" s="89" t="str"/>
-      <x:c r="F28" s="89" t="str"/>
-      <x:c r="G28" s="90" t="str"/>
+        <x:v>Portfolio Manager</x:v>
+      </x:c>
+      <x:c r="B28" s="85" t="str"/>
+      <x:c r="C28" s="86" t="str"/>
+      <x:c r="D28" s="86" t="str"/>
+      <x:c r="E28" s="86" t="str"/>
+      <x:c r="F28" s="86" t="str"/>
+      <x:c r="G28" s="87" t="str"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="114" t="str">
+        <x:v>Risk &amp; Derivatives</x:v>
+      </x:c>
+      <x:c r="B29" s="88" t="str"/>
+      <x:c r="C29" s="89" t="str"/>
+      <x:c r="D29" s="89" t="str"/>
+      <x:c r="E29" s="89" t="str"/>
+      <x:c r="F29" s="89" t="str"/>
+      <x:c r="G29" s="90" t="str"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="25" t="str">
         <x:v>Decision status</x:v>
       </x:c>
       <x:c r="B30" s="28" t="str">
-        <x:f>IF(COUNTIF(C25:C28,"Revise")+COUNTIF(C25:C28,"Reject")&gt;0,"REVISION REQUIRED",IF(COUNTIF(C25:C28,"Approve")=4,"APPROVED","INCOMPLETE"))</x:f>
+        <x:f>IF(COUNTIF(C25:C29,"Revise")+COUNTIF(C25:C29,"Reject")&gt;0,"REVISION REQUIRED",IF(COUNTIF(C25:C29,"Approve")=5,"APPROVED","INCOMPLETE"))</x:f>
         <x:v>INCOMPLETE</x:v>
       </x:c>
       <x:c r="C30" s="29"/>
@@ -5449,7 +5543,7 @@
     </x:row>
     <x:row r="44" ht="32" customHeight="1">
       <x:c r="A44" s="104" t="str">
-        <x:v>Approval requires four Approve votes. Any Revise or Reject vote produces REVISION REQUIRED; document the change and reconvene before the next gate.</x:v>
+        <x:v>Approval requires five Approve votes. Any Revise or Reject vote produces REVISION REQUIRED; document the change and reconvene before the next gate.</x:v>
       </x:c>
       <x:c r="B44" s="104"/>
       <x:c r="C44" s="104"/>
@@ -5489,7 +5583,7 @@
     <x:dataValidation type="list" sqref="G10:G15">
       <x:formula1>"Not reviewed,Reviewed,Needs follow-up"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="C25:C28">
+    <x:dataValidation type="list" sqref="C25:C29">
       <x:formula1>"Approve,Revise,Reject"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="E38:E42">

</xml_diff>